<commit_message>
style: beautify dashboards (CSFA, PTW, Workplan, Tools) with premium theme and layout alignment
</commit_message>
<xml_diff>
--- a/PPE dashboard/1-PPE_Detection_Report_v2.xlsx
+++ b/PPE dashboard/1-PPE_Detection_Report_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IITK pdfs\Acads\Intern stuff\Danone\Pojects Projects\Safety automation\Dashboards\PPE dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DC82B3B4-6907-4E2A-8AD8-7430EAE17D21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{08C7C8A8-9BD1-4C5D-AFC9-84A269E20D87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="3" r:id="rId1"/>
@@ -20492,9 +20492,9 @@
   <dimension ref="A1:W60"/>
   <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="46.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="38.42578125" customWidth="1"/>
     <col min="2" max="4" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" customWidth="1"/>
     <col min="6" max="6" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7" customWidth="1"/>
     <col min="8" max="8" width="7.7109375" customWidth="1"/>
@@ -20502,8 +20502,11 @@
     <col min="10" max="10" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="6.7109375" customWidth="1"/>
     <col min="12" max="13" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="6.85546875" customWidth="1"/>
     <col min="17" max="17" width="6.140625" customWidth="1"/>
     <col min="19" max="19" width="8.28515625" customWidth="1"/>
+    <col min="22" max="22" width="4.140625" customWidth="1"/>
+    <col min="23" max="23" width="6.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="15.6">
@@ -20642,7 +20645,9 @@
       <c r="V2" s="18">
         <v>7</v>
       </c>
-      <c r="W2" s="18"/>
+      <c r="W2" s="18">
+        <v>30</v>
+      </c>
     </row>
     <row r="3" spans="1:23">
       <c r="A3" s="6" t="s">
@@ -20711,7 +20716,9 @@
       <c r="V3" s="8">
         <v>7</v>
       </c>
-      <c r="W3" s="8"/>
+      <c r="W3" s="8">
+        <v>26</v>
+      </c>
     </row>
     <row r="4" spans="1:23">
       <c r="A4" s="6" t="s">
@@ -20746,7 +20753,9 @@
       <c r="V4" s="8">
         <v>1</v>
       </c>
-      <c r="W4" s="8"/>
+      <c r="W4" s="8">
+        <v>7</v>
+      </c>
     </row>
     <row r="5" spans="1:23">
       <c r="A5" s="6" t="s">
@@ -20809,7 +20818,9 @@
       <c r="V5" s="8">
         <v>2</v>
       </c>
-      <c r="W5" s="8"/>
+      <c r="W5" s="8">
+        <v>1</v>
+      </c>
     </row>
     <row r="6" spans="1:23">
       <c r="A6" s="6" t="s">
@@ -20862,7 +20873,9 @@
       </c>
       <c r="U6" s="8"/>
       <c r="V6" s="8"/>
-      <c r="W6" s="8"/>
+      <c r="W6" s="8">
+        <v>1</v>
+      </c>
     </row>
     <row r="7" spans="1:23">
       <c r="A7" s="6" t="s">
@@ -20986,7 +20999,9 @@
       <c r="V8" s="8">
         <v>6</v>
       </c>
-      <c r="W8" s="8"/>
+      <c r="W8" s="8">
+        <v>6</v>
+      </c>
     </row>
     <row r="9" spans="1:23">
       <c r="A9" s="6" t="s">
@@ -21055,7 +21070,9 @@
       <c r="V9" s="8">
         <v>5</v>
       </c>
-      <c r="W9" s="8"/>
+      <c r="W9" s="8">
+        <v>11</v>
+      </c>
     </row>
     <row r="10" spans="1:23">
       <c r="A10" s="6" t="s">
@@ -21177,7 +21194,9 @@
       <c r="V11" s="8">
         <v>6</v>
       </c>
-      <c r="W11" s="8"/>
+      <c r="W11" s="8">
+        <v>9</v>
+      </c>
     </row>
     <row r="12" spans="1:23">
       <c r="A12" s="6" t="s">
@@ -21316,7 +21335,9 @@
       <c r="V14" s="8">
         <v>2</v>
       </c>
-      <c r="W14" s="8"/>
+      <c r="W14" s="8">
+        <v>4</v>
+      </c>
     </row>
     <row r="15" spans="1:23">
       <c r="A15" s="6" t="s">
@@ -21379,7 +21400,9 @@
       <c r="V15" s="8">
         <v>4</v>
       </c>
-      <c r="W15" s="8"/>
+      <c r="W15" s="8">
+        <v>3</v>
+      </c>
     </row>
     <row r="16" spans="1:23">
       <c r="A16" s="6" t="s">
@@ -21446,7 +21469,9 @@
       <c r="V16" s="8">
         <v>5</v>
       </c>
-      <c r="W16" s="8"/>
+      <c r="W16" s="8">
+        <v>11</v>
+      </c>
     </row>
     <row r="17" spans="1:23">
       <c r="A17" s="6" t="s">
@@ -21513,7 +21538,9 @@
       <c r="V17" s="8">
         <v>41</v>
       </c>
-      <c r="W17" s="8"/>
+      <c r="W17" s="8">
+        <v>16</v>
+      </c>
     </row>
     <row r="18" spans="1:23" ht="15">
       <c r="A18" s="7" t="s">
@@ -21523,7 +21550,7 @@
         <v>316</v>
       </c>
       <c r="C18" s="7">
-        <f t="shared" ref="C18:V18" si="0">SUM(C2:C17)</f>
+        <f t="shared" ref="C18:W18" si="0">SUM(C2:C17)</f>
         <v>226</v>
       </c>
       <c r="D18" s="7">
@@ -21602,7 +21629,10 @@
         <f t="shared" si="0"/>
         <v>90</v>
       </c>
-      <c r="W18" s="8"/>
+      <c r="W18" s="29">
+        <f t="shared" si="0"/>
+        <v>125</v>
+      </c>
     </row>
     <row r="19" spans="1:23">
       <c r="E19" t="s">
@@ -21750,7 +21780,9 @@
       <c r="V22" s="18">
         <v>14</v>
       </c>
-      <c r="W22" s="18"/>
+      <c r="W22" s="18">
+        <v>10</v>
+      </c>
     </row>
     <row r="23" spans="1:23">
       <c r="A23" s="33" t="s">
@@ -21819,7 +21851,9 @@
       <c r="V23" s="8">
         <v>76</v>
       </c>
-      <c r="W23" s="8"/>
+      <c r="W23" s="8">
+        <v>115</v>
+      </c>
     </row>
     <row r="24" spans="1:23">
       <c r="A24" s="34" t="s">
@@ -21888,7 +21922,9 @@
       <c r="V24" s="22">
         <v>90</v>
       </c>
-      <c r="W24" s="22"/>
+      <c r="W24" s="22">
+        <v>125</v>
+      </c>
     </row>
     <row r="27" spans="1:23" ht="15.75">
       <c r="A27" s="32" t="s">
@@ -22047,7 +22083,9 @@
       <c r="V29" s="44">
         <v>1</v>
       </c>
-      <c r="W29" s="44"/>
+      <c r="W29" s="44">
+        <v>3</v>
+      </c>
     </row>
     <row r="30" spans="1:23">
       <c r="A30" s="6" t="s">
@@ -22112,7 +22150,9 @@
         <v>3</v>
       </c>
       <c r="V30" s="44"/>
-      <c r="W30" s="44"/>
+      <c r="W30" s="44">
+        <v>3</v>
+      </c>
     </row>
     <row r="31" spans="1:23">
       <c r="A31" s="6" t="s">
@@ -22173,7 +22213,9 @@
       <c r="V31" s="44">
         <v>1</v>
       </c>
-      <c r="W31" s="44"/>
+      <c r="W31" s="44">
+        <v>2</v>
+      </c>
     </row>
     <row r="32" spans="1:23">
       <c r="A32" s="6" t="s">
@@ -22292,7 +22334,9 @@
       <c r="T34" s="19"/>
       <c r="U34" s="44"/>
       <c r="V34" s="44"/>
-      <c r="W34" s="44"/>
+      <c r="W34" s="44">
+        <v>2</v>
+      </c>
     </row>
     <row r="35" spans="1:23">
       <c r="A35" s="20" t="s">
@@ -22321,7 +22365,9 @@
       <c r="T35" s="19"/>
       <c r="U35" s="44"/>
       <c r="V35" s="44"/>
-      <c r="W35" s="44"/>
+      <c r="W35" s="44">
+        <v>4</v>
+      </c>
     </row>
     <row r="36" spans="1:23">
       <c r="A36" s="23" t="s">
@@ -22414,7 +22460,9 @@
         <v>1</v>
       </c>
       <c r="V38" s="44"/>
-      <c r="W38" s="44"/>
+      <c r="W38" s="44">
+        <v>3</v>
+      </c>
     </row>
     <row r="39" spans="1:23">
       <c r="A39" s="6" t="s">
@@ -22483,7 +22531,9 @@
       <c r="V39" s="44">
         <v>82</v>
       </c>
-      <c r="W39" s="44"/>
+      <c r="W39" s="44">
+        <v>108</v>
+      </c>
     </row>
     <row r="40" spans="1:23">
       <c r="A40" s="20" t="s">
@@ -22576,8 +22626,12 @@
       <c r="U41" s="44">
         <v>109</v>
       </c>
-      <c r="V41" s="44"/>
-      <c r="W41" s="44"/>
+      <c r="V41" s="44">
+        <v>90</v>
+      </c>
+      <c r="W41" s="44">
+        <v>125</v>
+      </c>
     </row>
     <row r="44" spans="1:23">
       <c r="G44" t="s">
@@ -73695,6 +73749,9 @@
       <c r="A19" s="55">
         <v>46213</v>
       </c>
+      <c r="B19">
+        <v>293</v>
+      </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="55">
@@ -83626,6 +83683,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="8f6efb83-841f-4bde-8dcd-abbe1dde2f0d" xsi:nil="true"/>
@@ -83636,7 +83702,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D616D0BEE1F7064CB0A170B949FAEC87" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f7dad44da6bda0413aa3ad92c815d1ff">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b81dfca8-7f35-4830-97a6-0949ea5d014d" xmlns:ns3="8f6efb83-841f-4bde-8dcd-abbe1dde2f0d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="29141e1502a7a845c866280eabba5962" ns2:_="" ns3:_="">
     <xsd:import namespace="b81dfca8-7f35-4830-97a6-0949ea5d014d"/>
@@ -83849,25 +83915,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5C50E604-A3F5-4D3D-9E4A-DBB4802473BB}"/>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BC4AF886-44C2-4AAF-A02E-31D834BFAC77}"/>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C17D789-A193-4EB2-B6DE-D7FD358B037C}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5C50E604-A3F5-4D3D-9E4A-DBB4802473BB}"/>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>